<commit_message>
Updated port peripheral mappings.
</commit_message>
<xml_diff>
--- a/Design/port peripheral mapping.xlsx
+++ b/Design/port peripheral mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Hydra\Documents\DipTrace\Projects\MakerPnPControl\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE69C2A4-8F4F-421A-B0E6-59F2DE94EDDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC6D221-5394-4C86-B5B3-B77B4C476533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18165" yWindow="11970" windowWidth="23340" windowHeight="16140" xr2:uid="{C3A3646F-069D-4AE0-AC21-8ACD43A56D36}"/>
+    <workbookView xWindow="14475" yWindow="14790" windowWidth="23340" windowHeight="16140" xr2:uid="{C3A3646F-069D-4AE0-AC21-8ACD43A56D36}"/>
   </bookViews>
   <sheets>
     <sheet name="UFBGA176+25 Ports" sheetId="5" r:id="rId1"/>

</xml_diff>

<commit_message>
Move WIFI_INT2 to IO8. Fix using OCTOSPI2_NCS_2 for flash CS instead of OCTOSPIM_P2_NCS. Added OCTOSPI2_NCS2 to IO14 where the WIFI_INT2 was. Added *_NCS net suffixes to prevent further confusion.
* IO8 was unused anyway, except for boot control.
* H7, FPGA and C6 now can all read/write the flash.
* H7 can now correctly use OCTOSPI for the C6.
</commit_message>
<xml_diff>
--- a/Design/port peripheral mapping.xlsx
+++ b/Design/port peripheral mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Hydra\Documents\DipTrace\Projects\MakerPnPControl\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC6D221-5394-4C86-B5B3-B77B4C476533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4F2D4A-B682-44D8-9EBD-12BC5AE85E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14475" yWindow="14790" windowWidth="23340" windowHeight="16140" xr2:uid="{C3A3646F-069D-4AE0-AC21-8ACD43A56D36}"/>
+    <workbookView xWindow="24795" yWindow="12810" windowWidth="23340" windowHeight="16140" activeTab="1" xr2:uid="{C3A3646F-069D-4AE0-AC21-8ACD43A56D36}"/>
   </bookViews>
   <sheets>
     <sheet name="UFBGA176+25 Ports" sheetId="5" r:id="rId1"/>
@@ -2374,9 +2374,6 @@
     <t>OCTOSPI2_NCS_3</t>
   </si>
   <si>
-    <t>FLASH - NCS to flash</t>
-  </si>
-  <si>
     <t>EXPANSION_PORT</t>
   </si>
   <si>
@@ -2447,6 +2444,9 @@
   </si>
   <si>
     <t>TCXO, single pin</t>
+  </si>
+  <si>
+    <t>FLASH - NCS to flash and ESP32-C6 FSPIQ and FPGA SPI_SS_B</t>
   </si>
 </sst>
 </file>
@@ -5008,7 +5008,7 @@
         <v>725</v>
       </c>
       <c r="B47" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C47" t="s">
         <v>92</v>
@@ -5087,10 +5087,10 @@
         <v>726</v>
       </c>
       <c r="B49" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C49" t="s">
-        <v>768</v>
+        <v>792</v>
       </c>
       <c r="D49" s="1" t="e">
         <f>_xlfn.XLOOKUP(_xlfn.CONCAT("OCTOSPIM_",D$48),'UFBGA176+25 GPIOs'!$B$1:$B$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -5135,7 +5135,7 @@
         <v>766</v>
       </c>
       <c r="B50" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C50" t="s">
         <v>759</v>
@@ -5150,10 +5150,10 @@
         <v>767</v>
       </c>
       <c r="B51" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C51" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D51" s="1" t="str">
         <f>_xlfn.XLOOKUP($A51,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -5162,10 +5162,10 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B52" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C52" t="s">
         <v>92</v>
@@ -5177,7 +5177,7 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
@@ -5195,7 +5195,7 @@
         <v>149</v>
       </c>
       <c r="C55" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="D55" s="1" t="str">
         <f>_xlfn.XLOOKUP($A55,'UFBGA176+25 GPIOs'!$B$1:$B$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -6106,7 +6106,7 @@
         <v>374</v>
       </c>
       <c r="C95" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="D95" t="str" cm="1">
         <f t="array" ref="D95" xml:space="preserve"> IF(C95&lt;&gt;"",
@@ -6122,7 +6122,7 @@
         <v>99</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D96" t="str" cm="1">
         <f t="array" ref="D96" xml:space="preserve"> IF(C96&lt;&gt;"",
@@ -6145,7 +6145,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C98" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -6195,7 +6195,7 @@
         <v>106</v>
       </c>
       <c r="C105" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="D105" s="1" t="str">
         <f>_xlfn.XLOOKUP($A105,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -6207,7 +6207,7 @@
         <v>350</v>
       </c>
       <c r="C106" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D106" s="1" t="str">
         <f>_xlfn.XLOOKUP($A106,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -6219,7 +6219,7 @@
         <v>349</v>
       </c>
       <c r="C107" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="D107" s="1" t="str">
         <f>_xlfn.XLOOKUP($A107,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -6231,7 +6231,7 @@
         <v>351</v>
       </c>
       <c r="C108" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="D108" s="1" t="str">
         <f>_xlfn.XLOOKUP($A108,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -6243,7 +6243,7 @@
         <v>702</v>
       </c>
       <c r="C109" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="D109" s="1" t="str">
         <f>_xlfn.XLOOKUP($A109,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -6255,7 +6255,7 @@
         <v>700</v>
       </c>
       <c r="C110" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="D110" s="1" t="str">
         <f>_xlfn.XLOOKUP($A110,'UFBGA176+25 GPIOs'!$H$1:$H$133,'UFBGA176+25 GPIOs'!$A$1:$A$133)</f>
@@ -7932,7 +7932,7 @@
         <v>136</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="I52" s="1" t="b">
         <v>1</v>
@@ -7961,7 +7961,7 @@
         <v>136</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="I53" s="1" t="b">
         <v>1</v>
@@ -9763,7 +9763,7 @@
         <v>136</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="I119" s="1" t="b">
         <v>1</v>
@@ -10781,7 +10781,7 @@
         <v>461</v>
       </c>
       <c r="E36" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J36" t="s">
         <v>537</v>
@@ -10802,7 +10802,7 @@
         <v>462</v>
       </c>
       <c r="E37" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="J37" t="s">
         <v>537</v>
@@ -10813,7 +10813,7 @@
         <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C38">
         <f t="shared" si="0"/>
@@ -10826,7 +10826,7 @@
         <v>449</v>
       </c>
       <c r="F38" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="J38" t="s">
         <v>537</v>
@@ -10837,7 +10837,7 @@
         <v>28</v>
       </c>
       <c r="B39" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C39">
         <f t="shared" si="0"/>
@@ -10850,7 +10850,7 @@
         <v>92</v>
       </c>
       <c r="G39" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="J39" t="s">
         <v>537</v>
@@ -14687,7 +14687,7 @@
         <v>AMUX_EN</v>
       </c>
       <c r="C157" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
@@ -14696,7 +14696,7 @@
         <v>AMUX_A0</v>
       </c>
       <c r="C158" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
@@ -14705,7 +14705,7 @@
         <v>AMUX_A1</v>
       </c>
       <c r="C159" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>